<commit_message>
Update mining sector (factoriescap_s) 0.xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/mining sector (factoriescap_s) 0.xlsx
+++ b/clustering/sepsectors/mining sector (factoriescap_s) 0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="27">
   <si>
     <t>sector</t>
   </si>
@@ -91,6 +91,15 @@
   </si>
   <si>
     <t xml:space="preserve">Доли сквозных техн. и обучения персонала получены от ITcosts_s </t>
+  </si>
+  <si>
+    <t>верхний кластер:</t>
+  </si>
+  <si>
+    <t>нижний кластер:</t>
+  </si>
+  <si>
+    <t>разница</t>
   </si>
 </sst>
 </file>
@@ -100,7 +109,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -112,6 +121,8 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <sz val="11"/>
@@ -123,6 +134,15 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
@@ -165,7 +185,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -180,6 +200,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -483,7 +507,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="67" customWidth="1"/>
@@ -974,11 +998,764 @@
         <v>1.0604112949224313E-3</v>
       </c>
     </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D26" s="6">
+        <v>12596210.486</v>
+      </c>
+      <c r="E26" s="6">
+        <v>29618.176784399999</v>
+      </c>
+      <c r="F26" s="3">
+        <v>1.244197192428451E-3</v>
+      </c>
+      <c r="G26" s="3">
+        <v>9.1204876912707078E-4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D27" s="6">
+        <v>12460128.155999999</v>
+      </c>
+      <c r="E27" s="6">
+        <v>32672.95173072</v>
+      </c>
+      <c r="F27" s="3">
+        <v>2.8388815641284579E-2</v>
+      </c>
+      <c r="G27" s="3">
+        <v>1.009990774998547E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D28" s="6">
+        <v>11423484.0792</v>
+      </c>
+      <c r="E28" s="6">
+        <v>30582.725913679998</v>
+      </c>
+      <c r="F28" s="3">
+        <v>8.6595807302297054E-5</v>
+      </c>
+      <c r="G28" s="3">
+        <v>1.69804857508698E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D29" s="6">
+        <v>11300772.48</v>
+      </c>
+      <c r="E29" s="6">
+        <v>31974.339456000002</v>
+      </c>
+      <c r="F29" s="3">
+        <v>5.7574468505698965E-4</v>
+      </c>
+      <c r="G29" s="3">
+        <v>6.8807976565944413E-4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="6">
+        <f>AVERAGE(D26:D27)</f>
+        <v>12528169.320999999</v>
+      </c>
+      <c r="E31" s="6">
+        <f t="shared" ref="E31:G31" si="2">AVERAGE(E26:E27)</f>
+        <v>31145.56425756</v>
+      </c>
+      <c r="F31" s="3">
+        <f t="shared" si="2"/>
+        <v>1.4816506416856515E-2</v>
+      </c>
+      <c r="G31" s="3">
+        <f t="shared" si="2"/>
+        <v>9.6101977206280889E-4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D32" s="6">
+        <f>AVERAGE(D28:D29)</f>
+        <v>11362128.2796</v>
+      </c>
+      <c r="E32" s="6">
+        <f t="shared" ref="E32:G32" si="3">AVERAGE(E28:E29)</f>
+        <v>31278.53268484</v>
+      </c>
+      <c r="F32" s="3">
+        <f t="shared" si="3"/>
+        <v>3.3117024617964334E-4</v>
+      </c>
+      <c r="G32" s="3">
+        <f t="shared" si="3"/>
+        <v>1.193064170373212E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B34" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D34" s="6">
+        <f>D31/D32</f>
+        <v>1.1026252311808127</v>
+      </c>
+      <c r="E34" s="6">
+        <f t="shared" ref="E34:G34" si="4">E31/E32</f>
+        <v>0.99574889178403025</v>
+      </c>
+      <c r="F34" s="6">
+        <f t="shared" si="4"/>
+        <v>44.739847820807242</v>
+      </c>
+      <c r="G34" s="6">
+        <f t="shared" si="4"/>
+        <v>0.8055055175801521</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D37" s="6">
+        <v>1743254.7426</v>
+      </c>
+      <c r="E37" s="6">
+        <v>5649.2667995399997</v>
+      </c>
+      <c r="F37" s="3">
+        <v>4.3069526144492228E-2</v>
+      </c>
+      <c r="G37" s="3">
+        <v>2.415866866318173E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D38" s="6">
+        <v>1196714.5288</v>
+      </c>
+      <c r="E38" s="6">
+        <v>5296.7583626400001</v>
+      </c>
+      <c r="F38" s="3">
+        <v>0.1023070329623097</v>
+      </c>
+      <c r="G38" s="3">
+        <v>6.5499992306063972E-4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D39" s="6">
+        <v>1186586.3999999999</v>
+      </c>
+      <c r="E39" s="6">
+        <v>4305.8265600000004</v>
+      </c>
+      <c r="F39" s="3">
+        <v>7.4943726483957598E-2</v>
+      </c>
+      <c r="G39" s="3">
+        <v>1.251650972211942E-3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D40" s="6">
+        <v>1110225.9291999999</v>
+      </c>
+      <c r="E40" s="6">
+        <v>5731.3955529599998</v>
+      </c>
+      <c r="F40" s="3">
+        <v>2.961302102283718E-2</v>
+      </c>
+      <c r="G40" s="3">
+        <v>1.1157895805494109E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B42" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D42" s="6">
+        <f>AVERAGE(D37:D38)</f>
+        <v>1469984.6357</v>
+      </c>
+      <c r="E42" s="6">
+        <f t="shared" ref="E42:G42" si="5">AVERAGE(E37:E38)</f>
+        <v>5473.0125810899999</v>
+      </c>
+      <c r="F42" s="3">
+        <f t="shared" si="5"/>
+        <v>7.2688279553400958E-2</v>
+      </c>
+      <c r="G42" s="3">
+        <f t="shared" si="5"/>
+        <v>1.5354333946894063E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B43" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D43" s="6">
+        <f>AVERAGE(D39:D40)</f>
+        <v>1148406.1645999998</v>
+      </c>
+      <c r="E43" s="6">
+        <f t="shared" ref="E43:G43" si="6">AVERAGE(E39:E40)</f>
+        <v>5018.6110564800001</v>
+      </c>
+      <c r="F43" s="3">
+        <f t="shared" si="6"/>
+        <v>5.2278373753397389E-2</v>
+      </c>
+      <c r="G43" s="3">
+        <f t="shared" si="6"/>
+        <v>1.1837202763806765E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B45" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D45" s="6">
+        <f>D42/D43</f>
+        <v>1.2800215472650383</v>
+      </c>
+      <c r="E45" s="6">
+        <f t="shared" ref="E45:G45" si="7">E42/E43</f>
+        <v>1.090543283688677</v>
+      </c>
+      <c r="F45" s="6">
+        <f t="shared" si="7"/>
+        <v>1.3904082000767517</v>
+      </c>
+      <c r="G45" s="6">
+        <f t="shared" si="7"/>
+        <v>1.297125195307224</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C47" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D47" s="6">
+        <v>1730400.6762000001</v>
+      </c>
+      <c r="E47" s="6">
+        <v>11453.66344206</v>
+      </c>
+      <c r="F47" s="3">
+        <v>3.6351540108211508E-4</v>
+      </c>
+      <c r="G47" s="3">
+        <v>1.736681726385915E-4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C48" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D48" s="6">
+        <v>1665422.6664</v>
+      </c>
+      <c r="E48" s="6">
+        <v>8756.6848730599995</v>
+      </c>
+      <c r="F48" s="3">
+        <v>7.9418686213037007E-3</v>
+      </c>
+      <c r="G48" s="3">
+        <v>6.2767209962179716E-4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D49" s="6">
+        <v>1646977.0623999999</v>
+      </c>
+      <c r="E49" s="6">
+        <v>8501.7368701600008</v>
+      </c>
+      <c r="F49" s="3">
+        <v>3.13244725480416E-3</v>
+      </c>
+      <c r="G49" s="3">
+        <v>3.3557754651448161E-4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C50" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D50" s="6">
+        <v>1581936.48</v>
+      </c>
+      <c r="E50" s="6">
+        <v>7766.5038239999994</v>
+      </c>
+      <c r="F50" s="3">
+        <v>1.717868258658569E-2</v>
+      </c>
+      <c r="G50" s="3">
+        <v>1.213271790439538E-4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B52" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D52" s="6">
+        <f>AVERAGE(D47:D48)</f>
+        <v>1697911.6713</v>
+      </c>
+      <c r="E52" s="6">
+        <f t="shared" ref="E52:G52" si="8">AVERAGE(E47:E48)</f>
+        <v>10105.174157559999</v>
+      </c>
+      <c r="F52" s="3">
+        <f t="shared" si="8"/>
+        <v>4.1526920111929081E-3</v>
+      </c>
+      <c r="G52" s="3">
+        <f t="shared" si="8"/>
+        <v>4.0067013613019435E-4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B53" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D53" s="6">
+        <f>AVERAGE(D49:D50)</f>
+        <v>1614456.7711999998</v>
+      </c>
+      <c r="E53" s="6">
+        <f t="shared" ref="E53:G53" si="9">AVERAGE(E49:E50)</f>
+        <v>8134.1203470800001</v>
+      </c>
+      <c r="F53" s="3">
+        <f t="shared" si="9"/>
+        <v>1.0155564920694925E-2</v>
+      </c>
+      <c r="G53" s="3">
+        <f t="shared" si="9"/>
+        <v>2.2845236277921772E-4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B55" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D55" s="6">
+        <f>D52/D53</f>
+        <v>1.0516922481844897</v>
+      </c>
+      <c r="E55" s="6">
+        <f t="shared" ref="E55:G55" si="10">E52/E53</f>
+        <v>1.2423192338416251</v>
+      </c>
+      <c r="F55" s="6">
+        <f t="shared" si="10"/>
+        <v>0.40890802664562625</v>
+      </c>
+      <c r="G55" s="6">
+        <f t="shared" si="10"/>
+        <v>1.7538454461835107</v>
+      </c>
+    </row>
   </sheetData>
   <sortState ref="A2:G17">
     <sortCondition descending="1" ref="D2:D17"/>
   </sortState>
   <conditionalFormatting sqref="D2:D17">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E17">
+    <cfRule type="colorScale" priority="31">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F17">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G17">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D22:D23">
+    <cfRule type="colorScale" priority="28">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E22:E23">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F22:F23">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G22:G23">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D26:D29">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26:E29">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F26:F29">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G26:G29">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D31:D32">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E31:E32">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F31:F32">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G31:G32">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D37:D40">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E37:E40">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F37:F40">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G37:G40">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D42:D43">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E42:E43">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F42:F43">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G42:G43">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D47:D50">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -990,7 +1767,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E17">
+  <conditionalFormatting sqref="E47:E50">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -1002,7 +1779,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F17">
+  <conditionalFormatting sqref="F47:F50">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -1014,7 +1791,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G17">
+  <conditionalFormatting sqref="G47:G50">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -1026,7 +1803,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D22:D23">
+  <conditionalFormatting sqref="D52:D53">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -1038,7 +1815,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E22:E23">
+  <conditionalFormatting sqref="E52:E53">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1050,7 +1827,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F22:F23">
+  <conditionalFormatting sqref="F52:F53">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1062,7 +1839,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G22:G23">
+  <conditionalFormatting sqref="G52:G53">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>